<commit_message>
LMDI: Merge pull request #110 from folkehelseinstituttet/roar/fiks-oversettelsessjekk
Fiks oversettelsessjekk og rydd opp i byggkonfigurasjon ef179281898ec9ce1460957d465b374497b696f2
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-ingredient-strength.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-ingredient-strength.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="109">
   <si>
     <t>Property</t>
   </si>
@@ -84,7 +84,9 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Mengde ingrediens i det rekvirerte/administrerte legemidlet, angitt som Quantity eller som kode. Angir enten mengden virkestoff av ingrediensen i det rekvirerte/administrerte legemidlet (f.eks. 100 mg) eller hvilket volum av ingrediensen som er brukt for å produsere det rekvirerte/administrerte legemidlet (f.eks. 10 mL). Når volum benyttes skal ingredient.item angi «utgangslegemidlet» som ble brukt for å produsere det rekvirerte/administrerte legemidlet på en slik måte at «utgangslegemidlets» styrke kan utledes. Dette er nødvendig for å kunne beregne mengde virkestoff og styrke av ingrediensen i det rekvirerte/administrerte legemidlet.</t>
+    <t>Mengde ingrediens i det rekvirerte/administrerte legemidlet, angitt som Quantity eller som CodeableConcept.
+Ved Quantity: Enten mengden virkestoff av ingrediensen i det rekvirerte/administrerte legemidlet (f.eks. 100 mg) eller hvilket volum av ingrediensen som er brukt for å produsere det rekvirerte/administrerte legemidlet (f.eks. 10 mL). Når volum benyttes skal ingredient.item angi «utgangslegemidlet» som ble brukt for å produsere det rekvirerte/administrerte legemidlet på en slik måte at «utgangslegemidlets» styrke kan utledes. Dette er nødvendig for å kunne beregne mengde virkestoff og styrke av ingrediensen i det rekvirerte/administrerte legemidlet.
+Ved CodeableConcept: Kodet verdi som angir mengden ingrediens, f.eks. qs eller trace. F.eks. fra kodeverk "Angi at bestanddel i legemiddelblanding ikke har eksakt mengde" (OID 7502) eller "Medication-ingredientstrength" http://hl7.org/fhir/CodeSystem/medication-ingredientstrength</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -344,13 +346,7 @@
     <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
   </si>
   <si>
-    <t>preferred</t>
-  </si>
-  <si>
-    <t>Medication Ingredient Strength Codes</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/medication-ingredientstrength</t>
+    <t>Ved kodet mengde anbefales det norske kodeverket med OID 2.16.578.1.12.4.1.1.7502, eller kodeverket medication-ingredientstrength fra FHIR R5 (kodene qs og trace).</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
@@ -699,8 +695,8 @@
     <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="30.75" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="46.5390625" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="18.49609375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="16.828125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
@@ -1276,7 +1272,9 @@
       <c r="M6" t="s" s="2">
         <v>106</v>
       </c>
-      <c r="N6" s="2"/>
+      <c r="N6" t="s" s="2">
+        <v>107</v>
+      </c>
       <c r="O6" s="2"/>
       <c r="P6" t="s" s="2">
         <v>77</v>
@@ -1301,13 +1299,13 @@
         <v>77</v>
       </c>
       <c r="X6" t="s" s="2">
-        <v>107</v>
+        <v>77</v>
       </c>
       <c r="Y6" t="s" s="2">
-        <v>108</v>
+        <v>77</v>
       </c>
       <c r="Z6" t="s" s="2">
-        <v>109</v>
+        <v>77</v>
       </c>
       <c r="AA6" t="s" s="2">
         <v>77</v>
@@ -1337,7 +1335,7 @@
         <v>77</v>
       </c>
       <c r="AJ6" t="s" s="2">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="AK6" t="s" s="2">
         <v>102</v>

</xml_diff>